<commit_message>
Documentacion de Elegir perfil y del espacio del profesional (DAS v1.15, CP-050 a CP-060, defectos 15 a 24)
DAS: decisiones D25 (reemplaza D21), D26 y D27, flujo del espacio del profesional, Ilustraciones 6 y 10 nuevas. Planilla: 11 casos ejecutados contra el backend y MySQL reales y notas en los casos desactualizados. Registro de defectos 15 a 24. Capturas evidencia_14 a evidencia_22 y mockups del PO.
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Plan de Pruebas/Registro_Defectos.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Plan de Pruebas/Registro_Defectos.xlsx
@@ -392,7 +392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I1000"/>
+  <dimension ref="A1:I1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="9.380000000000001" customWidth="1" style="9" min="1" max="1"/>
@@ -1018,105 +1018,405 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="3" t="n"/>
-      <c r="C17" s="3" t="n"/>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3" t="n"/>
-      <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="5" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="3" t="n"/>
-      <c r="C18" s="3" t="n"/>
-      <c r="D18" s="3" t="n"/>
-      <c r="E18" s="3" t="n"/>
-      <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="5" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="3" t="n"/>
-      <c r="C19" s="3" t="n"/>
-      <c r="D19" s="3" t="n"/>
-      <c r="E19" s="3" t="n"/>
-      <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="5" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="3" t="n"/>
-      <c r="C20" s="3" t="n"/>
-      <c r="D20" s="3" t="n"/>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="5" t="n"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1" s="9">
-      <c r="B21" s="3" t="n"/>
-      <c r="C21" s="3" t="n"/>
-      <c r="D21" s="3" t="n"/>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="7" t="n"/>
-    </row>
-    <row r="22" ht="15.75" customHeight="1" s="9">
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="5" t="n"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1" s="9">
-      <c r="B23" s="3" t="n"/>
-      <c r="C23" s="3" t="n"/>
-      <c r="D23" s="3" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="5" t="n"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1" s="9">
-      <c r="B24" s="3" t="n"/>
-      <c r="C24" s="3" t="n"/>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="5" t="n"/>
-    </row>
-    <row r="25" ht="15.75" customHeight="1" s="9">
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="5" t="n"/>
-    </row>
-    <row r="26" ht="15.75" customHeight="1" s="9">
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="5" t="n"/>
+    <row r="17" s="9">
+      <c r="B17" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>N/A (revisión de código del PR #11)</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Backend y frontend - profesionales</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Al integrar main en la rama del PR #11 quedaron versiones antiguas de los archivos de profesionales: se perdían la búsqueda avanzada, la ficha por id, los filtros y las reseñas (FS-HU-22 a FS-HU-24), el backend no arrancaba y el build del frontend fallaba.</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Grave</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 04-10-2026 al revisar el PR #11 (32 pruebas del frontend y 10 suites del backend fallaban). Luis Méndez lo corrigió en el PR #12 el 07-10-2026, que reemplazó al PR #11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" s="9">
+      <c r="B18" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>CP-060 (ficha propia)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Backend - profesionales</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>En el PR #12, guardar la ficha propia solo actualizaba una fila existente de profesionales y, si no existía, lanzaba un error: todo profesional nuevo recibía "Ocurrió un error inesperado" (500) al guardar su ficha.</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>Grave</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 07-10-2026 al revisar el PR #12 (5 cuentas profesionales locales sin fila). Corregido el mismo día en el commit 84716a4: la ficha se crea o se actualiza (upsert; DAS, D27). Fusionado con el PR #12 el 08-10-2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" s="9">
+      <c r="B19" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>CP-057 (validación de la ficha)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Backend - profesionales</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>En el PR #12, PUT /api/profesionales/mi-ficha no usaba su validador: aceptaba especialidad vacía o coordenadas fuera de rango. Además existía un POST /mi-ficha que no hacía falta.</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Seguridad</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 07-10-2026 al revisar el PR #12 (una prueba automatizada esperaba 400 y recibía 200). Corregido en el commit 84716a4: el PUT valida la especialidad del catálogo, la comuna, la modalidad y la ubicación, y se quitó el POST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" s="9">
+      <c r="B20" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>N/A (revisión de código del PR #12)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Configuración</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>El PR #12 eliminaba backend/.env.example y frontend/.env.example, las plantillas para configurar el proyecto en un equipo nuevo.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Configuración</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 07-10-2026 al revisar el PR #12. Restaurados en el commit 84716a4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" s="9">
+      <c r="B21" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>N/A (revisión de código del PR #12)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Frontend - perfil</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Con el PR #12 el aviso de cuenta creada o de sesión iniciada aparecía dos veces en "Mi perfil": lo mostraban el diseño común y la página.</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Interfaz</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Leve</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 07-10-2026 al revisar el PR #12. Corregido en el commit 84716a4: solo lo muestra el diseño común (DisenoAplicacion).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" s="9">
+      <c r="B22" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>CP-051 (Continuar como usuario)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Frontend - Elegir perfil</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Al elegir "Usuario" en "Elegir perfil" se abría el Inicio en vez del asistente de perfil.</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 08-10-2026 por la prueba automatizada de Elegir perfil, antes de entregar el cambio. El usuario sigue con su asistente (/perfil) y el profesional va a su Inicio.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" s="9">
+      <c r="B23" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>CP-052 (Continuar como profesional)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Frontend - Elegir perfil</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Al elegir "Profesional", el aviso "¡Listo! Tu cuenta profesional está creada" se borraba antes de llegar al Inicio del profesional.</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Leve</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 08-10-2026 por la prueba automatizada de Elegir perfil. La pantalla solo descarta el aviso que había al llegar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" s="9">
+      <c r="B24" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>CP-054 (separación por rol)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Frontend - navegación</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Con una sesión guardada antes del cambio (sin el dato rolConfirmado) y una cuenta que aún no elegía su perfil, el Inicio y "Elegir perfil" podían redirigirse entre sí sin fin.</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Funcional</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Medio</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 08-10-2026 por la prueba automatizada del asistente. Cuando la API indica que falta elegir el perfil, se corrige la sesión guardada y la ruta protegida lleva a "Elegir perfil".</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" s="9">
+      <c r="B25" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>CP-056 (revisión visual)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Frontend - menú del profesional</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>En el menú del profesional el ícono del lema se veía gigante y las etiquetas "Próximamente" se cortaban porque el menú se desbordaba.</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Interfaz</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Leve</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 08-10-2026 al revisar el Inicio del profesional en el navegador. El ícono tiene tamaño fijo y en ese menú "Próximamente" se muestra como un punto naranja (el texto sigue disponible para lectores de pantalla).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" s="9">
+      <c r="B26" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>CP-050 (revisión visual)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Frontend - Elegir perfil</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>El adorno de la esquina superior tapaba parte del logo.</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Interfaz</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Leve</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 08-10-2026 en el navegador. El adorno se achicó y en celular se oculta.</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="9">
       <c r="B27" s="3" t="n"/>

</xml_diff>

<commit_message>
Defecto 36 y CP-109: modelo de Groq openai/gpt-oss-120b y asistente probado con Groq real
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Plan de Pruebas/Registro_Defectos.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Plan de Pruebas/Registro_Defectos.xlsx
@@ -392,7 +392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I1000"/>
+  <dimension ref="A1:I1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="9.380000000000001" customWidth="1" style="9" min="1" max="1"/>
@@ -1881,13 +1881,46 @@
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="9">
-      <c r="B38" s="1" t="n"/>
-      <c r="C38" s="1" t="n"/>
-      <c r="D38" s="1" t="n"/>
-      <c r="E38" s="1" t="n"/>
-      <c r="F38" s="1" t="n"/>
-      <c r="G38" s="1" t="n"/>
-      <c r="H38" s="1" t="n"/>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>CP-109</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Backend - asistente IA</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Con la clave real de Groq, cada mensaje al asistente terminaba en «El asistente no está disponible en este momento»: el modelo configurado por defecto (llama-3.3-70b-versatile) ya no existe en Groq y el proveedor respondía 404 (model_not_found).</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Configuración</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Grave</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Corregido</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Detectado el 22-10-2026 por Rodrigo Cárcamo al ejecutar CP-109 con la clave real. Corregido el mismo día: el modelo por defecto pasa a openai/gpt-oss-120b (config/env.js y .env.example), elegido entre los modelos de texto activos de la cuenta (openai/gpt-oss-120b, openai/gpt-oss-20b y qwen/qwen3.8-27b) por la calidad de sus respuestas en español, en alrededor de 1 s. IA_MODELO permite cambiarlo sin tocar el código si Groq vuelve a retirar un modelo. Verificado con CP-109 (6/6).</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="9">
       <c r="B39" s="1" t="n"/>

</xml_diff>

<commit_message>
Defecto 39: revision de Luis Mendez, ajuste del cambio de dia y fusion de los PR 29 y 30
</commit_message>
<xml_diff>
--- a/FASE 2/Evidencias Proyecto/Evidencias de documentación/Plan de Pruebas/Registro_Defectos.xlsx
+++ b/FASE 2/Evidencias Proyecto/Evidencias de documentación/Plan de Pruebas/Registro_Defectos.xlsx
@@ -392,7 +392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1000"/>
+  <dimension ref="B1:I1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="9.380000000000001" customWidth="1" style="9" min="1" max="1"/>
@@ -2044,7 +2044,7 @@
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>Informado el 23-10-2026 por Nicolás Silva en la revisión del PR #29 (cambios solicitados). Corregido el mismo día en feat/asistente-ia: el mensaje se reserva antes de llamar al proveedor con un solo UPDATE condicionado (mensajes &lt; límite) o un INSERT, y si el proveedor o el guardado fallan el cupo se devuelve. Pruebas de Jest con tres solicitudes simultáneas al iniciar y al continuar, y verificación contra MySQL real. Verificado con CP-122 (backend 304/304).</t>
+          <t>Informado el 23-10-2026 por Luis Méndez en la revisión del PR #29 (cambios solicitados). Corregido el mismo día en feat/asistente-ia: el mensaje se reserva antes de llamar al proveedor con un solo UPDATE condicionado (mensajes &lt; límite) o un INSERT, y si el proveedor o el guardado fallan el cupo se devuelve. Pruebas de Jest con tres solicitudes simultáneas al iniciar y al continuar, y verificación contra MySQL real. Verificado con CP-122 (backend 304/304). Al revisar, Luis Méndez agregó que el reinicio de día solo avance a un día posterior (una solicitud tardía del día anterior ya no reinicia el contador del día nuevo) y la comprobación npm run test:mysql:asistente (23 condiciones, todas aprobadas; Plan de Pruebas/Asistente_Cupo_MySQL*). PR #29 y #30 aprobados por Luis y fusionados en main el 23-10-2026.</t>
         </is>
       </c>
     </row>

</xml_diff>